<commit_message>
Updates as I fixing figures
</commit_message>
<xml_diff>
--- a/03. Results/SpatialResult - Tax rich.xlsx
+++ b/03. Results/SpatialResult - Tax rich.xlsx
@@ -1,76 +1,83 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\00. GitHub_Projects\Invert_Diversity_Poato\03. Results\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_C2CE303C64B1A95F5178811D060A53129275A060" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t xml:space="preserve">field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">statistic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S2_F6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DHARMa Moran's I test for distance-based autocorrelation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S3_F7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S4_F8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S4_F9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S5_F8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S6_F10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S6_F11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S6_F8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S7_F10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S7_F12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S8_F10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S8_F13</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>statistic</t>
+  </si>
+  <si>
+    <t>p_value</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>S2_F6</t>
+  </si>
+  <si>
+    <t>DHARMa Moran's I test for distance-based autocorrelation</t>
+  </si>
+  <si>
+    <t>S3_F7</t>
+  </si>
+  <si>
+    <t>S4_F8</t>
+  </si>
+  <si>
+    <t>S4_F9</t>
+  </si>
+  <si>
+    <t>S5_F8</t>
+  </si>
+  <si>
+    <t>S6_F10</t>
+  </si>
+  <si>
+    <t>S6_F11</t>
+  </si>
+  <si>
+    <t>S6_F8</t>
+  </si>
+  <si>
+    <t>S7_F10</t>
+  </si>
+  <si>
+    <t>S7_F12</t>
+  </si>
+  <si>
+    <t>S8_F10</t>
+  </si>
+  <si>
+    <t>S8_F13</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -106,6 +113,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -387,11 +403,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -405,169 +421,169 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="n">
-        <v>-0.0349823823700049</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.695418222642751</v>
+      <c r="B2">
+        <v>-3.4982382370004901E-2</v>
+      </c>
+      <c r="C2">
+        <v>0.69541822264275099</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="n">
-        <v>-0.0200624838748171</v>
-      </c>
-      <c r="C3" t="n">
+      <c r="B3">
+        <v>-2.00624838748171E-2</v>
+      </c>
+      <c r="C3">
         <v>0.557972796865572</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="n">
-        <v>-0.0219868957350651</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.456738306832166</v>
+      <c r="B4">
+        <v>-2.1986895735065098E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.45673830683216599</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="n">
-        <v>-0.0601495161284711</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.601380180459281</v>
+      <c r="B5">
+        <v>-6.0149516128471102E-2</v>
+      </c>
+      <c r="C5">
+        <v>0.60138018045928099</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="n">
-        <v>-0.0906835941526912</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.346995985192882</v>
+      <c r="B6">
+        <v>-9.0683594152691199E-2</v>
+      </c>
+      <c r="C6">
+        <v>0.34699598519288199</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="n">
-        <v>-0.14663405468881</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.590134287868915</v>
+      <c r="B7">
+        <v>-0.14663405468880999</v>
+      </c>
+      <c r="C7">
+        <v>0.59013428786891498</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" t="n">
-        <v>-0.0367296089471249</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.0485412812334287</v>
+      <c r="B8">
+        <v>-3.6729608947124903E-2</v>
+      </c>
+      <c r="C8">
+        <v>4.8541281233428699E-2</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="n">
-        <v>-0.0341040417061767</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.646083606292473</v>
+      <c r="B9">
+        <v>-3.4104041706176702E-2</v>
+      </c>
+      <c r="C9">
+        <v>0.64608360629247297</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" t="n">
-        <v>-0.146598712738174</v>
-      </c>
-      <c r="C10" t="n">
+      <c r="B10">
+        <v>-0.14659871273817399</v>
+      </c>
+      <c r="C10">
         <v>0.60408583768641</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="n">
-        <v>-0.0712262867710571</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.585493670032274</v>
+      <c r="B11">
+        <v>-7.1226286771057107E-2</v>
+      </c>
+      <c r="C11">
+        <v>0.58549367003227404</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" t="n">
-        <v>-0.117178947788047</v>
-      </c>
-      <c r="C12" t="n">
+      <c r="B12">
+        <v>-0.11717894778804699</v>
+      </c>
+      <c r="C12">
         <v>0.922352608977278</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" t="n">
-        <v>-0.0311499814792124</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.863903689427497</v>
+      <c r="B13">
+        <v>-3.1149981479212399E-2</v>
+      </c>
+      <c r="C13">
+        <v>0.86390368942749696</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
@@ -575,6 +591,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>